<commit_message>
fix bug of change shift admin
</commit_message>
<xml_diff>
--- a/exports/shifts_report.xlsx
+++ b/exports/shifts_report.xlsx
@@ -467,7 +467,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hossein Karimi</t>
+          <t>--- خالی ---</t>
         </is>
       </c>
     </row>
@@ -487,7 +487,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ali Ahmadi، Hossein Karimi</t>
+          <t>--- خالی ---</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add and remove negahban
</commit_message>
<xml_diff>
--- a/exports/shifts_report.xlsx
+++ b/exports/shifts_report.xlsx
@@ -447,7 +447,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>--- خالی ---</t>
+          <t>نگهبان، نگهبان، نگهبان</t>
         </is>
       </c>
     </row>
@@ -457,7 +457,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>--- خالی ---</t>
+          <t>نگهبان</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>--- خالی ---</t>
+          <t>نگهبان</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>--- خالی ---</t>
+          <t>محمدرضا قنبری</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>--- خالی ---</t>
+          <t>محمدرضا قنبری</t>
         </is>
       </c>
     </row>
@@ -557,7 +557,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>--- خالی ---</t>
+          <t>محمدرضا قنبری</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>--- خالی ---</t>
+          <t>پویا هارونی</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>--- خالی ---</t>
+          <t>علی عبدالهی، محمدرضا قنبری</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>--- خالی ---</t>
+          <t>پویا هارونی</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>--- خالی ---</t>
+          <t>پویا هارونی</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>--- خالی ---</t>
+          <t>پویا هارونی، نگهبان</t>
         </is>
       </c>
     </row>

</xml_diff>